<commit_message>
Agrego admin error fecha
Agrego la vista admin en donde solventa el error que no se veía la fecha
</commit_message>
<xml_diff>
--- a/tareas_export.xlsx
+++ b/tareas_export.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +41,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00343A40"/>
         <bgColor rgb="00343A40"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0028A745"/>
+        <bgColor rgb="0028A745"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC107"/>
+        <bgColor rgb="00FFC107"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,9 +74,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -432,17 +453,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -484,6 +505,190 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>IFCT163PO</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>INTELIGENCIA ARTIFICIAL APLICADA A LA EMPRESA</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>FEVECTA 2026</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-09</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>admin@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>FCOM01</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>MANIPULADOR DE ALIMENTOS</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>FEVECTA 2026</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>admin@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>ADGG020PO</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>EXCEL AVANZADO</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>FEVECTA 2026</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>admin@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>COMT104PO</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>BLOG PARA LA COMUNICACIÓN DE NEGOCIOS</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>FEVECTA 2026</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>admin@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>paco</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>paco</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>paco</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Paco</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>paco@gmail.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
font-size:12px y cambio en el tamaño del form
</commit_message>
<xml_diff>
--- a/tareas_export.xlsx
+++ b/tareas_export.xlsx
@@ -453,17 +453,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="53" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -510,26 +510,26 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>IFCT163PO</t>
+          <t>Practica 1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>INTELIGENCIA ARTIFICIAL APLICADA A LA EMPRESA</t>
+          <t>enfrente alberto practica1/pr.mt.2026</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>FEVECTA 2026</t>
+          <t>Practicas</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2025-12-09</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -539,35 +539,39 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>practicas</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>admin@correo.com</t>
+          <t>practica@nomail.com</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>FCOM01</t>
+          <t>Practicas 2</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>MANIPULADOR DE ALIMENTOS</t>
+          <t>Al lado de Pablo practica5/pr.mt.2026</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>FEVECTA 2026</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
+          <t>Practicas</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Completada</t>
@@ -575,71 +579,79 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>practicas</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>admin@correo.com</t>
+          <t>practica@nomail.com</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ADGG020PO</t>
+          <t>Practica 3</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>EXCEL AVANZADO</t>
+          <t>Al lado de Rodrigo practica3/pr.mt.2026</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>FEVECTA 2026</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Completada</t>
+          <t>Practicas</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>practicas</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>admin@correo.com</t>
+          <t>practica@nomail.com</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>COMT104PO</t>
+          <t>Practica 4</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>BLOG PARA LA COMUNICACIÓN DE NEGOCIOS</t>
+          <t>Al lado de Ricardo practica4/pr.mt.2026</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>FEVECTA 2026</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+          <t>Practicas</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Pendiente</t>
@@ -647,48 +659,612 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>practicas</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>admin@correo.com</t>
+          <t>practica@nomail.com</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Practica 5</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Al lado de Barbara practica2/pr.mt.2026</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Practicas</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>practicas</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>practica@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Practica 6</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Al lado de Ruth practica6/pr.mt.2026</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Practicas</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>practicas</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>practica@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Practica 7</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Al lado de Sara practica7/pr.mt.2026</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Practicas</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>practicas</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>practica@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Practica 8</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Al lado de Ines practica8/pr.mt.2026</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Practicas</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>practicas</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>practica@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Practica 9</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Al lado de no se sabe  practica9/pr.mt.2026</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Practicas</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>practicas</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>practica@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>COMT095PO Rocio Ortega</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>MEC id=3691 // FORMACIÓN MBS id=182</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>F24</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>clonacion</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>clonacion@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>HOTA0003 Xiana</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>MEC id=5268 // FORMACIÓN MBS id=183</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>F24</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>clonacion</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>clonacion@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>HOTA0003 Xiana</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>MEC id=5268 // CONFEMETAL id=132</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>F24</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>clonacion</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>clonacion@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>HOTA0003 Xiana</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MEC id=5268 //  FESMC id=412</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>F24</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>clonacion</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>clonacion@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>QUIE022PO</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>IP_2026_REVERTE</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Licencias</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>licencias</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>licencias@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>MEC</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Elena Carré Otero</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>rrhh@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>MBS</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Alfonso Claro Casanova</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>rrhh@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>MEC</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Marta Palomares Rúa</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>rrhh@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>paco</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>paco</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>paco</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Paco</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>paco@gmail.com</t>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>FFC</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Begoña González Pardo</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>rrhh@nomail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>SEAD071PO Teri</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Poner licencias y quitar exámenes, cambiar scorm</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Pedagogia</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>clonacion</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>clonacion@nomail.com</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrego una nueva hoja en excel con las tareas en el día y un reporte general
</commit_message>
<xml_diff>
--- a/tareas_export.xlsx
+++ b/tareas_export.xlsx
@@ -612,9 +612,9 @@
           <t>2026-02-20</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -652,9 +652,9 @@
           <t>2026-02-23</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -732,9 +732,9 @@
           <t>2026-02-27</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">

</xml_diff>